<commit_message>
Lab 2 review fixes: rename test package, P note for 5.2, readable sheet headers
</commit_message>
<xml_diff>
--- a/lab2/out/lab2_estimation_model.xlsx
+++ b/lab2/out/lab2_estimation_model.xlsx
@@ -3182,7 +3182,7 @@
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>Feature complete: системне і навантажувальне тестування</t>
+          <t>Системне і навантажувальне тестування</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
@@ -3792,7 +3792,7 @@
     <col width="7" customWidth="1" min="6" max="6"/>
     <col width="7" customWidth="1" min="7" max="7"/>
     <col width="7" customWidth="1" min="8" max="8"/>
-    <col width="10" customWidth="1" min="9" max="9"/>
+    <col width="13" customWidth="1" min="9" max="9"/>
     <col width="60" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
@@ -4036,7 +4036,7 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Feature complete: системне і навантажувальне тестування</t>
+          <t>Системне і навантажувальне тестування</t>
         </is>
       </c>
       <c r="C6" s="6">
@@ -4067,7 +4067,11 @@
         <f>'WBS і CPM'!W17</f>
         <v/>
       </c>
-      <c r="J6" s="2" t="inlineStr"/>
+      <c r="J6" s="2" t="inlineStr">
+        <is>
+          <t>P = 16: повторний прогін навантажувального тесту k6 після оптимізації агрегатів F9 і повторна перевірка критеріїв F1...F11 після виправлень</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Lab 2 review fixes: package 1.2 and 3.2 P notes match appendix, partial A5 check before start, workbook start note
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/lab2/out/lab2_estimation_model.xlsx
+++ b/lab2/out/lab2_estimation_model.xlsx
@@ -627,7 +627,7 @@
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>після тестів A1, A2, A5 з ЛР № 1</t>
+          <t>після тестів A1, A2 і часткової перевірки A5 з ЛР № 1</t>
         </is>
       </c>
     </row>
@@ -3889,7 +3889,7 @@
       </c>
       <c r="J2" s="2" t="inlineStr">
         <is>
-          <t>ключова невизначеність варіанта: карта регістрів Modbus надходить від постачальника лічильників (A12), частина лічильників відповідає нестабільно; у P закладено 2 ітерації очікування по 5 робочих днів</t>
+          <t>ключова невизначеність варіанта: карта регістрів Modbus надходить від постачальника лічильників (A12), частина лічильників відповідає нестабільно; у P закладено 2 ітерації очікування по 5 робочих днів і 2 дні повторного тесту зчитування</t>
         </is>
       </c>
     </row>
@@ -3979,7 +3979,7 @@
       </c>
       <c r="J4" s="2" t="inlineStr">
         <is>
-          <t>поріг max(3σ; 10%) може потребувати 2...3 циклів налаштування на розмічених даних (A7)</t>
+          <t>поріг max(3σ; 10%) може потребувати 3 додаткових циклів налаштування на розмічених даних (A7)</t>
         </is>
       </c>
     </row>

</xml_diff>